<commit_message>
fix YHAAO-1204: 资产信息导入导出的功能修改,revert template
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/asset/assetImport/APM_Asset_TieFaces_Template.xlsx
+++ b/src/src/main/webapp/portal/asset/assetImport/APM_Asset_TieFaces_Template.xlsx
@@ -113,7 +113,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>tie:each(items="assetList", var="asset")</t>
+          <t>tie:each(items="assetList", var="asset", length="1" allowAdd="False")</t>
         </r>
       </text>
     </comment>
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="548">
   <si>
     <t>设备列表</t>
   </si>
@@ -518,6 +518,24 @@
       <t>设备型号</t>
     </r>
     <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>XXXX</t>
+  </si>
+  <si>
+    <t>XXX医疗器械有限公司</t>
+  </si>
+  <si>
+    <t>XX医疗设备有限公司</t>
+  </si>
+  <si>
+    <t>XXX</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
+    <t>平均年限</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -810,6 +828,10 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
+    <t>放射科</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
     <t>眼科手术用其他器械</t>
   </si>
   <si>
@@ -1941,6 +1963,12 @@
   </si>
   <si>
     <t>非计量设备</t>
+  </si>
+  <si>
+    <t>急救设备</t>
+  </si>
+  <si>
+    <t>二级</t>
   </si>
   <si>
     <t>医用CT</t>
@@ -2321,6 +2349,10 @@
   </si>
   <si>
     <t>设备分类</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>张三</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
@@ -4946,7 +4978,7 @@
     <col min="53" max="53" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:53" ht="27" customHeight="1">
+    <row r="1" spans="1:53" ht="27">
       <c r="A1" s="24" t="s">
         <v>43</v>
       </c>
@@ -4955,7 +4987,7 @@
       </c>
       <c r="C1" s="24"/>
       <c r="D1" s="123" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E1" s="124"/>
       <c r="F1" s="124"/>
@@ -4974,7 +5006,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="D2" s="124"/>
       <c r="E2" s="124"/>
@@ -5057,8 +5089,14 @@
       <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:53" ht="21">
-      <c r="A5" s="120"/>
-      <c r="B5" s="121"/>
+      <c r="A5" s="120">
+        <f>COUNTA('Asset List'!$B$7:$B$100)</f>
+        <v>1</v>
+      </c>
+      <c r="B5" s="121">
+        <f>SUM('Asset List'!$Y$7:$Y$100)</f>
+        <v>0</v>
+      </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="11"/>
@@ -5078,43 +5116,43 @@
         <v>111</v>
       </c>
       <c r="E6" s="118" t="s">
-        <v>524</v>
+        <v>534</v>
       </c>
       <c r="F6" s="29" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="G6" s="30" t="s">
-        <v>513</v>
+        <v>523</v>
       </c>
       <c r="H6" s="30" t="s">
         <v>33</v>
       </c>
       <c r="I6" s="30" t="s">
-        <v>523</v>
+        <v>533</v>
       </c>
       <c r="J6" s="30" t="s">
-        <v>525</v>
+        <v>535</v>
       </c>
       <c r="K6" s="31" t="s">
         <v>112</v>
       </c>
       <c r="L6" s="32" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="M6" s="30" t="s">
-        <v>510</v>
+        <v>520</v>
       </c>
       <c r="N6" s="93" t="s">
-        <v>511</v>
+        <v>521</v>
       </c>
       <c r="O6" s="93" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="P6" s="30" t="s">
         <v>36</v>
       </c>
       <c r="Q6" s="30" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="R6" s="30" t="s">
         <v>113</v>
@@ -5126,7 +5164,7 @@
         <v>86</v>
       </c>
       <c r="U6" s="30" t="s">
-        <v>522</v>
+        <v>532</v>
       </c>
       <c r="V6" s="30" t="s">
         <v>38</v>
@@ -5150,7 +5188,7 @@
         <v>21</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>526</v>
+        <v>536</v>
       </c>
       <c r="AD6" s="30" t="s">
         <v>23</v>
@@ -5159,10 +5197,10 @@
         <v>24</v>
       </c>
       <c r="AF6" s="93" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="AG6" s="93" t="s">
-        <v>512</v>
+        <v>522</v>
       </c>
       <c r="AH6" s="30" t="s">
         <v>26</v>
@@ -5186,77 +5224,105 @@
         <v>32</v>
       </c>
       <c r="AO6" s="32" t="s">
-        <v>488</v>
+        <v>497</v>
       </c>
       <c r="AP6" s="32" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="AQ6" s="32" t="s">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="AR6" s="32" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="AS6" s="32" t="s">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="AT6" s="32" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="AU6" s="32" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="AV6" s="32" t="s">
-        <v>495</v>
+        <v>504</v>
       </c>
       <c r="AW6" s="32" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="AX6" s="109" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="AY6" s="32" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="AZ6" s="32" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="BA6" s="109" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
     </row>
     <row r="7" spans="1:53" ht="15.75">
       <c r="A7" s="35" t="s">
-        <v>536</v>
+        <v>546</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>537</v>
-      </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="110"/>
-      <c r="E7" s="34"/>
+        <v>547</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="D7" s="110" t="s">
+        <v>519</v>
+      </c>
+      <c r="E7" s="34" t="s">
+        <v>9</v>
+      </c>
       <c r="F7" s="34"/>
-      <c r="G7" s="94"/>
-      <c r="H7" s="37"/>
+      <c r="G7" s="94" t="s">
+        <v>178</v>
+      </c>
+      <c r="H7" s="37" t="s">
+        <v>115</v>
+      </c>
       <c r="I7" s="37"/>
       <c r="J7" s="37"/>
       <c r="K7" s="16"/>
-      <c r="L7" s="28"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
+      <c r="L7" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>259</v>
+      </c>
+      <c r="O7" s="17" t="s">
+        <v>426</v>
+      </c>
       <c r="P7" s="17"/>
       <c r="Q7" s="17"/>
-      <c r="R7" s="28"/>
-      <c r="S7" s="28"/>
+      <c r="R7" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="S7" s="28" t="s">
+        <v>118</v>
+      </c>
       <c r="T7" s="17"/>
       <c r="U7" s="17"/>
       <c r="V7" s="28"/>
       <c r="W7" s="17"/>
       <c r="X7" s="17"/>
-      <c r="Y7" s="36"/>
-      <c r="Z7" s="18"/>
-      <c r="AA7" s="36"/>
+      <c r="Y7" s="36">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="18">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="36" t="s">
+        <v>119</v>
+      </c>
       <c r="AB7" s="19"/>
       <c r="AC7" s="20"/>
       <c r="AD7" s="21"/>
@@ -5275,14 +5341,30 @@
       <c r="AQ7" s="114"/>
       <c r="AR7" s="114"/>
       <c r="AS7" s="114"/>
-      <c r="AT7" s="23"/>
-      <c r="AU7" s="23"/>
-      <c r="AV7" s="23"/>
-      <c r="AW7" s="23"/>
-      <c r="AX7" s="23"/>
-      <c r="AY7" s="23"/>
-      <c r="AZ7" s="23"/>
-      <c r="BA7" s="23"/>
+      <c r="AT7" s="23" t="s">
+        <v>429</v>
+      </c>
+      <c r="AU7" s="23" t="s">
+        <v>439</v>
+      </c>
+      <c r="AV7" s="23" t="s">
+        <v>449</v>
+      </c>
+      <c r="AW7" s="23" t="s">
+        <v>445</v>
+      </c>
+      <c r="AX7" s="23" t="s">
+        <v>452</v>
+      </c>
+      <c r="AY7" s="23" t="s">
+        <v>448</v>
+      </c>
+      <c r="AZ7" s="23" t="s">
+        <v>441</v>
+      </c>
+      <c r="BA7" s="23" t="s">
+        <v>542</v>
+      </c>
     </row>
     <row r="8" spans="1:53" s="105" customFormat="1" ht="15.75">
       <c r="A8" s="35"/>
@@ -10400,6 +10482,9 @@
       <c r="BA100" s="23"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D1:L2"/>
+  </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="D1 E4:F6 P7:R7">
     <cfRule type="expression" dxfId="107" priority="79">
@@ -11110,7 +11195,7 @@
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="119" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="11" spans="1:1">
@@ -11545,7 +11630,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" thickBot="1">
       <c r="A1" s="125" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B1" s="125"/>
       <c r="C1" s="125"/>
@@ -11553,16 +11638,16 @@
     </row>
     <row r="2" spans="1:4" ht="17.25" thickBot="1">
       <c r="A2" s="58" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B2" s="59" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C2" s="59" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D2" s="59" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16.5">
@@ -11570,11 +11655,11 @@
         <v>1</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="C3" s="62"/>
       <c r="D3" s="63" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17.25" thickBot="1">
@@ -11582,11 +11667,11 @@
         <v>2</v>
       </c>
       <c r="B4" s="65" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C4" s="66"/>
       <c r="D4" s="67" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="71" customFormat="1" ht="17.25" thickBot="1">
@@ -11597,7 +11682,7 @@
     </row>
     <row r="6" spans="1:4" s="71" customFormat="1" ht="16.5" thickBot="1">
       <c r="A6" s="126" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B6" s="127"/>
       <c r="C6" s="127"/>
@@ -11605,16 +11690,16 @@
     </row>
     <row r="7" spans="1:4" s="71" customFormat="1" ht="17.25" thickBot="1">
       <c r="A7" s="72" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B7" s="73" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D7" s="73" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16.5">
@@ -11622,7 +11707,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="75" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C8" s="76"/>
       <c r="D8" s="77"/>
@@ -11632,7 +11717,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="61" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C9" s="78"/>
       <c r="D9" s="79"/>
@@ -11642,7 +11727,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="61" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C10" s="78"/>
       <c r="D10" s="79"/>
@@ -11652,7 +11737,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="61" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C11" s="78"/>
       <c r="D11" s="79"/>
@@ -11662,7 +11747,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="61" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C12" s="78"/>
       <c r="D12" s="79"/>
@@ -11672,7 +11757,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="61" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C13" s="78"/>
       <c r="D13" s="79"/>
@@ -11682,7 +11767,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="78" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C14" s="78"/>
       <c r="D14" s="79"/>
@@ -11692,7 +11777,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="61" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C15" s="78"/>
       <c r="D15" s="79"/>
@@ -11702,11 +11787,11 @@
         <v>11</v>
       </c>
       <c r="B16" s="61" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C16" s="78"/>
       <c r="D16" s="79" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="16.5">
@@ -11714,7 +11799,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="61" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C17" s="78"/>
       <c r="D17" s="79"/>
@@ -11724,7 +11809,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="61" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C18" s="78"/>
       <c r="D18" s="79"/>
@@ -11734,7 +11819,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="61" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C19" s="78"/>
       <c r="D19" s="79"/>
@@ -11744,7 +11829,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="61" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C20" s="78"/>
       <c r="D20" s="79"/>
@@ -11754,7 +11839,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="65" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C21" s="80"/>
       <c r="D21" s="81"/>
@@ -11764,7 +11849,7 @@
     </row>
     <row r="23" spans="1:4" ht="16.5" thickBot="1">
       <c r="A23" s="129" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B23" s="130"/>
       <c r="C23" s="130"/>
@@ -11772,16 +11857,16 @@
     </row>
     <row r="24" spans="1:4" ht="17.25" thickBot="1">
       <c r="A24" s="83" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B24" s="84" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C24" s="84" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D24" s="84" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="16.5" thickBot="1">
@@ -11789,11 +11874,11 @@
         <v>17</v>
       </c>
       <c r="B25" s="85" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C25" s="86"/>
       <c r="D25" s="87" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="16.5" thickBot="1">
@@ -11801,11 +11886,11 @@
         <v>18</v>
       </c>
       <c r="B26" s="85" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="C26" s="62"/>
       <c r="D26" s="63" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -11813,11 +11898,11 @@
         <v>19</v>
       </c>
       <c r="B27" s="85" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C27" s="88"/>
       <c r="D27" s="89" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="16.5" thickBot="1">
@@ -11825,11 +11910,11 @@
         <v>20</v>
       </c>
       <c r="B28" s="90" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C28" s="91"/>
       <c r="D28" s="92" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -11864,23 +11949,23 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="132" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B1" s="132" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C1" s="132"/>
       <c r="D1" s="132" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="132"/>
       <c r="B2" s="38" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D2" s="132"/>
     </row>
@@ -11890,7 +11975,7 @@
       </c>
       <c r="B3" s="40"/>
       <c r="C3" s="40" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D3" s="41"/>
     </row>
@@ -11899,10 +11984,10 @@
         <v>13</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D4" s="41"/>
     </row>
@@ -11916,19 +12001,19 @@
     </row>
     <row r="6" spans="1:4" ht="16.5">
       <c r="A6" s="45" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B6" s="44"/>
       <c r="C6" s="44" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="D6" s="41" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16.5">
       <c r="A7" s="43" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B7" s="46"/>
       <c r="C7" s="46"/>
@@ -11936,11 +12021,11 @@
     </row>
     <row r="8" spans="1:4" ht="16.5">
       <c r="A8" s="45" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B8" s="47"/>
       <c r="C8" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D8" s="41"/>
     </row>
@@ -11950,19 +12035,19 @@
       </c>
       <c r="B9" s="47"/>
       <c r="C9" s="47" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D9" s="49" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16.5">
       <c r="A10" s="45" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B10" s="47"/>
       <c r="C10" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D10" s="41"/>
     </row>
@@ -11980,7 +12065,7 @@
       </c>
       <c r="B12" s="47"/>
       <c r="C12" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D12" s="41"/>
     </row>
@@ -11989,10 +12074,10 @@
         <v>35</v>
       </c>
       <c r="B13" s="47" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C13" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D13" s="41"/>
     </row>
@@ -12006,11 +12091,11 @@
     </row>
     <row r="15" spans="1:4" ht="16.5">
       <c r="A15" s="45" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B15" s="47"/>
       <c r="C15" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D15" s="41"/>
     </row>
@@ -12024,11 +12109,11 @@
     </row>
     <row r="17" spans="1:4" ht="16.5">
       <c r="A17" s="45" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B17" s="47"/>
       <c r="C17" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D17" s="41"/>
     </row>
@@ -12038,7 +12123,7 @@
       </c>
       <c r="B18" s="47"/>
       <c r="C18" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D18" s="41"/>
     </row>
@@ -12056,7 +12141,7 @@
       </c>
       <c r="B20" s="47"/>
       <c r="C20" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D20" s="41"/>
     </row>
@@ -12066,7 +12151,7 @@
       </c>
       <c r="B21" s="47"/>
       <c r="C21" s="47" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D21" s="41"/>
     </row>
@@ -12124,7 +12209,7 @@
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D28" s="41"/>
     </row>
@@ -12134,7 +12219,7 @@
       </c>
       <c r="B29" s="47"/>
       <c r="C29" s="47" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D29" s="41"/>
     </row>
@@ -12188,44 +12273,44 @@
     </row>
     <row r="36" spans="1:4" ht="16.5">
       <c r="A36" s="50" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B36" s="51"/>
       <c r="C36" s="51" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D36" s="41"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="52" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="53"/>
       <c r="B40" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C40" s="54" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="55"/>
       <c r="B41" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C41" s="54" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="56"/>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C42" s="54" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -12270,472 +12355,472 @@
   <sheetData>
     <row r="1" spans="1:13" s="27" customFormat="1">
       <c r="A1" s="96" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>35</v>
       </c>
       <c r="C1" s="96" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="D1" s="96" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="E1" s="96" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="F1" s="96" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="G1" s="96" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="H1" s="96" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="I1" s="100" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="J1" s="102" t="s">
-        <v>485</v>
+        <v>494</v>
       </c>
       <c r="K1" s="104" t="s">
-        <v>486</v>
+        <v>495</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>487</v>
+        <v>496</v>
       </c>
       <c r="M1" s="122" t="s">
-        <v>531</v>
+        <v>541</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="95" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="B2" s="107" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="C2" s="95" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="D2" s="95" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="E2" s="98" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="F2" s="107" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="G2" s="97" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="H2" s="95" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="I2" s="99" t="s">
-        <v>441</v>
+        <v>450</v>
       </c>
       <c r="J2" s="101" t="s">
-        <v>472</v>
+        <v>481</v>
       </c>
       <c r="K2" s="103" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
       <c r="L2" s="107" t="s">
-        <v>479</v>
+        <v>488</v>
       </c>
       <c r="M2" s="116" t="s">
-        <v>532</v>
+        <v>542</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17.25" customHeight="1">
       <c r="A3" s="95" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="B3" s="107" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C3" s="95" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="D3" s="95" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="E3" s="98" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="F3" s="107" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="G3" s="97" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="H3" s="95" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="I3" s="99" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
       <c r="J3" s="101" t="s">
-        <v>473</v>
+        <v>482</v>
       </c>
       <c r="K3" s="103" t="s">
-        <v>477</v>
+        <v>486</v>
       </c>
       <c r="L3" s="107" t="s">
-        <v>480</v>
+        <v>489</v>
       </c>
       <c r="M3" s="116" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="95" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="B4" s="107" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="C4" s="95" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="D4" s="95" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="E4" s="98" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="F4" s="107" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="G4" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="H4" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="I4" s="99" t="s">
-        <v>443</v>
+        <v>452</v>
       </c>
       <c r="J4" s="101" t="s">
-        <v>474</v>
+        <v>483</v>
       </c>
       <c r="K4" s="103" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="L4" s="107" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="M4" s="116" t="s">
-        <v>534</v>
+        <v>544</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="95" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="B5" s="107" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C5" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="D5" s="95" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="E5" s="98" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="F5" s="107" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="I5" s="99" t="s">
-        <v>444</v>
+        <v>453</v>
       </c>
       <c r="J5" s="101" t="s">
-        <v>475</v>
+        <v>484</v>
       </c>
       <c r="K5" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="L5" s="107" t="s">
-        <v>482</v>
+        <v>491</v>
       </c>
       <c r="M5" s="116" t="s">
-        <v>474</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="116" t="s">
-        <v>517</v>
+        <v>527</v>
       </c>
       <c r="B6" s="116" t="s">
-        <v>517</v>
+        <v>527</v>
       </c>
       <c r="D6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="E6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="F6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="I6" s="99" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
       <c r="J6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="L6" s="107" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="M6" s="116" t="s">
-        <v>473</v>
+        <v>482</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="116" t="s">
-        <v>518</v>
+        <v>528</v>
       </c>
       <c r="B7" s="116" t="s">
-        <v>518</v>
+        <v>528</v>
       </c>
       <c r="I7" s="99" t="s">
-        <v>446</v>
+        <v>455</v>
       </c>
       <c r="L7" s="107" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="M7" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="116" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="B8" s="116" t="s">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="I8" s="99" t="s">
-        <v>447</v>
+        <v>456</v>
       </c>
       <c r="L8" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="95" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="B9" s="107" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="I9" s="99" t="s">
-        <v>448</v>
+        <v>457</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="95" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="B10" s="107" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="I10" s="99" t="s">
-        <v>449</v>
+        <v>458</v>
       </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="117" t="s">
-        <v>516</v>
+        <v>526</v>
       </c>
       <c r="B11" s="117" t="s">
-        <v>516</v>
+        <v>526</v>
       </c>
       <c r="H11" s="107"/>
       <c r="I11" s="99" t="s">
-        <v>450</v>
+        <v>459</v>
       </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="117" t="s">
-        <v>520</v>
+        <v>530</v>
       </c>
       <c r="B12" s="117" t="s">
-        <v>520</v>
+        <v>530</v>
       </c>
       <c r="H12" s="107"/>
       <c r="I12" s="99" t="s">
-        <v>451</v>
+        <v>460</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="117" t="s">
-        <v>521</v>
+        <v>531</v>
       </c>
       <c r="B13" s="117" t="s">
-        <v>521</v>
+        <v>531</v>
       </c>
       <c r="H13" s="107"/>
       <c r="I13" s="99" t="s">
-        <v>452</v>
+        <v>461</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="95" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="B14" s="107" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="H14" s="107"/>
       <c r="I14" s="99" t="s">
-        <v>453</v>
+        <v>462</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="B15" s="116"/>
       <c r="H15" s="107"/>
       <c r="I15" s="99" t="s">
-        <v>454</v>
+        <v>463</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="B16" s="107"/>
       <c r="H16" s="107"/>
       <c r="I16" s="99" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="107"/>
       <c r="H17" s="107"/>
       <c r="I17" s="99" t="s">
-        <v>456</v>
+        <v>465</v>
       </c>
     </row>
     <row r="18" spans="2:9">
       <c r="B18" s="107"/>
       <c r="H18" s="107"/>
       <c r="I18" s="99" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="107"/>
       <c r="H19" s="107"/>
       <c r="I19" s="99" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="107"/>
       <c r="H20" s="107"/>
       <c r="I20" s="99" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="107"/>
       <c r="H21" s="107"/>
       <c r="I21" s="99" t="s">
-        <v>460</v>
+        <v>469</v>
       </c>
     </row>
     <row r="22" spans="2:9">
       <c r="B22" s="107"/>
       <c r="H22" s="107"/>
       <c r="I22" s="99" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
     </row>
     <row r="23" spans="2:9">
       <c r="B23" s="107"/>
       <c r="H23" s="107"/>
       <c r="I23" s="99" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
     </row>
     <row r="24" spans="2:9">
       <c r="B24" s="107"/>
       <c r="H24" s="107"/>
       <c r="I24" s="99" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
     </row>
     <row r="25" spans="2:9">
       <c r="B25" s="107"/>
       <c r="H25" s="107"/>
       <c r="I25" s="99" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
     </row>
     <row r="26" spans="2:9">
       <c r="H26" s="107"/>
       <c r="I26" s="99" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
     </row>
     <row r="27" spans="2:9">
       <c r="H27" s="107"/>
       <c r="I27" s="99" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
     </row>
     <row r="28" spans="2:9">
       <c r="H28" s="107"/>
       <c r="I28" s="99" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" spans="2:9">
       <c r="H29" s="107"/>
       <c r="I29" s="99" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
     </row>
     <row r="30" spans="2:9">
       <c r="H30" s="107"/>
       <c r="I30" s="99" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
     </row>
     <row r="31" spans="2:9">
       <c r="H31" s="107"/>
       <c r="I31" s="99" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
     </row>
     <row r="32" spans="2:9">
       <c r="H32" s="107"/>
       <c r="I32" s="99" t="s">
-        <v>470</v>
+        <v>479</v>
       </c>
     </row>
     <row r="33" spans="8:9">
       <c r="H33" s="107"/>
       <c r="I33" s="99" t="s">
-        <v>471</v>
+        <v>480</v>
       </c>
     </row>
     <row r="34" spans="8:9">
       <c r="H34" s="107"/>
       <c r="I34" s="115" t="s">
-        <v>514</v>
+        <v>524</v>
       </c>
     </row>
     <row r="35" spans="8:9">
       <c r="I35" s="115" t="s">
-        <v>515</v>
+        <v>525</v>
       </c>
     </row>
     <row r="36" spans="8:9">
       <c r="I36" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
   </sheetData>
@@ -12928,10 +13013,10 @@
   <sheetData>
     <row r="1" spans="1:41">
       <c r="A1" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="B1" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C1" t="s">
         <v>46</v>
@@ -12946,7 +13031,7 @@
         <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="H1" t="s">
         <v>50</v>
@@ -12961,7 +13046,7 @@
         <v>53</v>
       </c>
       <c r="L1" t="s">
-        <v>528</v>
+        <v>538</v>
       </c>
       <c r="M1" t="s">
         <v>54</v>
@@ -12994,7 +13079,7 @@
         <v>63</v>
       </c>
       <c r="W1" t="s">
-        <v>529</v>
+        <v>539</v>
       </c>
       <c r="X1" t="s">
         <v>64</v>
@@ -13048,884 +13133,884 @@
         <v>80</v>
       </c>
       <c r="AO1" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="2" spans="1:41">
       <c r="A2" s="95" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B2" s="95" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="C2" s="95" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="D2" s="95" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="E2" s="95" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="F2" s="95" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="G2" s="95" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="H2" s="95" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="I2" s="95" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="J2" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="K2" s="95" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="L2" s="95" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="M2" s="95" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="N2" s="95" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="O2" s="95" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="P2" s="95" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="Q2" s="95" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="R2" s="95" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="S2" s="95" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="T2" s="95" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="U2" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="V2" s="95" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="W2" s="95" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="X2" s="95" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="Y2" s="95" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="Z2" s="95" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="AA2" s="95" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="AB2" s="95" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="AC2" s="95" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="AD2" s="95" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="AE2" s="95" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="AF2" s="95" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="AG2" s="95" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="AH2" s="95" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="AI2" s="95" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="AJ2" s="95" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="AK2" s="95" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="AL2" s="95" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="AM2" s="95" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="AN2" s="95" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
     </row>
     <row r="3" spans="1:41">
       <c r="A3" s="95" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="B3" s="95" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C3" s="95" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="D3" s="95" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="E3" s="95" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="F3" s="95" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="G3" s="95" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="H3" s="95" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="I3" s="95" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="K3" s="95" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="L3" s="95" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="M3" s="95" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="N3" s="95" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="O3" s="95" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="P3" s="95" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="Q3" s="95" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="R3" s="95" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="S3" s="95" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="T3" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="U3" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="V3" s="95" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="W3" s="95" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="X3" s="95" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="Y3" s="95" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="Z3" s="95" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="AA3" s="95" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="AB3" s="95" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="AC3" s="95" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="AD3" s="95" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="AE3" s="95" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="AF3" s="95" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="AG3" s="95" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="AH3" s="95" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="AI3" s="95" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="AJ3" s="95" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="AK3" s="95" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="AL3" s="95" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="AM3" s="95" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="AN3" s="95" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" spans="1:41">
       <c r="A4" s="95" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B4" s="95" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C4" s="95" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="D4" s="95" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="E4" s="95" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="F4" s="95" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="G4" s="95" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="H4" s="95" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="I4" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="K4" s="95" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="L4" s="95" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="M4" s="95" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="N4" s="95" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="O4" s="95" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="P4" s="95" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="Q4" s="95" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="R4" s="95" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="S4" s="95" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="U4" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="V4" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="W4" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="X4" s="95" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="Y4" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="Z4" s="95" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="AA4" s="95" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="AB4" s="95" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="AC4" s="95" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="AD4" s="95" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="AE4" s="95" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="AF4" s="95" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="AG4" s="95" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="AH4" s="95" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="AI4" s="95" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="AJ4" s="95" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="AK4" s="95" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="AL4" s="95" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="AM4" s="95" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="AN4" s="95" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
     </row>
     <row r="5" spans="1:41">
       <c r="A5" s="95" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B5" s="95" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C5" s="95" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="D5" s="95" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="E5" s="95" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="F5" s="95" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="G5" s="95" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="H5" s="95" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="K5" s="95" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="L5" s="95" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="M5" s="95" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="N5" s="95" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="O5" s="95" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="P5" s="95" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="Q5" s="95" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="R5" s="95" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="S5" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="U5" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="V5" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="X5" s="95" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="Z5" s="95" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="AA5" s="95" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="AB5" s="95" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="AC5" s="95" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="AD5" s="95" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="AE5" s="95" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="AF5" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AG5" s="95" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="AH5" s="95" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="AI5" s="95" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="AJ5" s="95" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="AK5" s="95" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="AL5" s="95" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="AM5" s="95" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="AN5" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="6" spans="1:41">
       <c r="A6" s="95" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B6" s="95" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C6" s="95" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="D6" s="95" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="E6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="F6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="G6" s="95" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="H6" s="95" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="K6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="L6" s="95" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="M6" s="95" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="N6" s="95" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="O6" s="95" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="P6" s="95" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="Q6" s="95" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="R6" s="95" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="U6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="V6" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="X6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="Z6" s="95" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="AA6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AB6" s="95" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="AC6" s="95" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="AD6" s="95" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="AE6" s="95" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="AG6" s="95" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="AH6" s="95" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="AI6" s="95" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="AJ6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AK6" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AL6" s="95" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="AM6" s="95" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
     </row>
     <row r="7" spans="1:41">
       <c r="A7" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="B7" s="95" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C7" s="95" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="D7" s="95" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="G7" s="95" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="H7" s="95" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="L7" s="95" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="M7" s="95" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="N7" s="95" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="O7" s="95" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="P7" s="95" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="Q7" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="R7" s="95" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="V7" s="95" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="Z7" s="95" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="AB7" s="95" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="AC7" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AD7" s="95" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="AE7" s="95" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="AG7" s="95" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="AH7" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AI7" s="95" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="AL7" s="95" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="AM7" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="8" spans="1:41">
       <c r="B8" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="C8" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="D8" s="95" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="G8" s="95" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="H8" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="L8" s="95" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="M8" s="95" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="N8" s="95" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="O8" s="95" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="P8" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="R8" s="95" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="V8" s="95" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="Z8" s="95" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="AB8" s="95" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="AD8" s="95" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="AE8" s="95" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="AG8" s="95" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="AI8" s="95" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="AL8" s="95" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
     </row>
     <row r="9" spans="1:41">
       <c r="D9" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="G9" s="95" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="L9" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="M9" s="95" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="N9" s="95" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="O9" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="R9" s="95" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="V9" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="Z9" s="95" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="AB9" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AD9" s="95" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="AE9" s="95" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="AG9" s="95" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="AI9" s="95" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="AL9" s="95" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
     </row>
     <row r="10" spans="1:41">
       <c r="G10" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="M10" s="95" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="N10" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="R10" s="95" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="Z10" s="95" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="AD10" s="95" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="AE10" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AG10" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AI10" s="95" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="AL10" s="95" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
     </row>
     <row r="11" spans="1:41">
       <c r="M11" s="95" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="R11" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="Z11" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AD11" s="95" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="AI11" s="95" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="AL11" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="12" spans="1:41">
       <c r="M12" s="95" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="AD12" s="95" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="AI12" s="95" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13" spans="1:41">
       <c r="M13" s="95" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="AD13" s="95" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="AI13" s="95" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
     </row>
     <row r="14" spans="1:41">
       <c r="M14" s="95" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="AD14" s="95" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="AI14" s="95" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
     </row>
     <row r="15" spans="1:41">
       <c r="M15" s="95" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="AD15" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
       <c r="AI15" s="95" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16" spans="1:41">
       <c r="M16" s="95" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="AI16" s="95" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
     </row>
     <row r="17" spans="13:35">
       <c r="M17" s="95" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="AI17" s="95" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
     </row>
     <row r="18" spans="13:35">
       <c r="M18" s="95" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="AI18" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
     <row r="19" spans="13:35">
       <c r="M19" s="95" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" spans="13:35">
       <c r="M20" s="95" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
     </row>
     <row r="21" spans="13:35">
       <c r="M21" s="116" t="s">
-        <v>527</v>
+        <v>537</v>
       </c>
     </row>
   </sheetData>

</xml_diff>